<commit_message>
feat(templates): add the slice board sheet to engineering_tracker.xlsx
ticket-tracker.md 定義了切片看板的契約，但範本沒有那張表——契約指向一個不存在
的工作表，等於沒有落地。

engineering_tracker.xlsx 新增「③ 切片看板」，沿用既有兩張表的視覺慣例：
紫色 ID 欄、橙色來源欄（來源SCN）、灰色內容欄、綠色狀態與證據欄，粗體表頭、
凍結 B2、一列範例、狀態下拉（待開始/進行中/待驗證/完成/封鎖）到第 500 列。
封面補一行說明前緣定義與併發規則的出處。

既有的①規格追溯與②模組BOM未動（dimension 與資料驗證均驗證過）。

順帶把文件裡的「③切片看板」統一為「③ 切片看板」——①② 都有空格，工作表名
不一致會讓依名稱定位的腳本抓不到。

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RcSZBFeFs1mpRYTrXWKFHY
</commit_message>
<xml_diff>
--- a/VibeCoding_Workflow_Templates/03_architecture/engineering_tracker.xlsx
+++ b/VibeCoding_Workflow_Templates/03_architecture/engineering_tracker.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="封面" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="① 規格追溯" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="② 模組BOM" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="③ 切片看板" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -39,7 +40,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -64,6 +65,30 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E4DFEC"/>
+        <bgColor rgb="00E4DFEC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+        <bgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+        <bgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -93,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -110,6 +135,18 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -475,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -488,6 +525,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -495,6 +533,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -502,6 +541,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -513,6 +553,13 @@
       <c r="A8" t="inlineStr">
         <is>
           <t>橙色欄＝來源ID（指向上游檔）。狀態滾動更新，不必一開始填滿。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>③ 切片看板：/deliver 的 SLC-* 交付切片狀態機。前緣＝狀態「待開始」且未認領且所有 Blocked by 已完成。併發寫入規則見 docs/document-system/ticket-tracker.md §6（唯一寫入者）。</t>
         </is>
       </c>
     </row>
@@ -755,4 +802,119 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>切片ID</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>標題</t>
+        </is>
+      </c>
+      <c r="C1" s="10" t="inlineStr">
+        <is>
+          <t>來源SCN</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>接縫</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>Blocked by</t>
+        </is>
+      </c>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t>狀態</t>
+        </is>
+      </c>
+      <c r="G1" s="11" t="inlineStr">
+        <is>
+          <t>認領者</t>
+        </is>
+      </c>
+      <c r="H1" s="11" t="inlineStr">
+        <is>
+          <t>認領時間</t>
+        </is>
+      </c>
+      <c r="I1" s="11" t="inlineStr">
+        <is>
+          <t>證據</t>
+        </is>
+      </c>
+      <c r="J1" s="9" t="inlineStr">
+        <is>
+          <t>備註</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SLC-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>結帳可送出並收到確認</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>SCN-003, SCN-004</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>OrderService.submit</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>待開始</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>先做 prefactor：抽出 PriceCalc</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="F2:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"待開始,進行中,待驗證,完成,封鎖"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>